<commit_message>
Add longitudinal MAP data regression analysis and charts
</commit_message>
<xml_diff>
--- a/data/2024_2025 MAP Data.xlsx
+++ b/data/2024_2025 MAP Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b669fe2ece5530df/NWMSU/DATA ANALYTICS FUNDAMENTALS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\map-regression\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{545419B2-D4C0-4730-9050-A0F35CCE6FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFD7A1CA-A328-4C4E-A39D-D27981293367}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA6D1FE-A71C-4D1D-AE49-16F5FC3A13F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22180" windowHeight="14860" xr2:uid="{449B78BD-E0C3-49C0-8A5B-B657B24BCA65}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="3">
   <si>
     <t>Algebra 1</t>
   </si>
@@ -47,10 +47,7 @@
     <t>Geometry</t>
   </si>
   <si>
-    <t>RitScore F24</t>
-  </si>
-  <si>
-    <t>Geometry F24</t>
+    <t>RitScore</t>
   </si>
 </sst>
 </file>
@@ -437,15 +434,12 @@
   <dimension ref="A1:G131"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>

</xml_diff>